<commit_message>
include TP-Link Archer C7
</commit_message>
<xml_diff>
--- a/nbench/list2026.xlsx
+++ b/nbench/list2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\archive\github\benchmark\nbench\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50C9BA65-6DF8-4DC5-AC07-62E853870D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E47D8A1-FAEC-44A2-A457-7A44A36D207F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6990" yWindow="30" windowWidth="26505" windowHeight="15705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1730" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1731" uniqueCount="269">
   <si>
     <t>CPU</t>
   </si>
@@ -849,6 +849,9 @@
   </si>
   <si>
     <t>6.12.74, gcc 14.3.0</t>
+  </si>
+  <si>
+    <t>__Integer Index__</t>
   </si>
 </sst>
 </file>
@@ -937,7 +940,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1028,18 +1031,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF6F8FA"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -1084,7 +1075,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1154,6 +1145,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1166,31 +1160,19 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="10" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="10" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -1652,7 +1634,7 @@
       <c r="J2" s="13">
         <v>40892</v>
       </c>
-      <c r="K2" s="41" t="s">
+      <c r="K2" s="37" t="s">
         <v>228</v>
       </c>
       <c r="M2" s="18">
@@ -1783,7 +1765,7 @@
       <c r="J4" s="13">
         <v>41487</v>
       </c>
-      <c r="K4" s="41" t="s">
+      <c r="K4" s="37" t="s">
         <v>228</v>
       </c>
       <c r="M4" s="18">
@@ -1849,7 +1831,7 @@
       <c r="J5" s="13">
         <v>41489</v>
       </c>
-      <c r="K5" s="39" t="s">
+      <c r="K5" s="35" t="s">
         <v>229</v>
       </c>
       <c r="M5" s="18">
@@ -1915,7 +1897,7 @@
       <c r="J6" s="13">
         <v>41122</v>
       </c>
-      <c r="K6" s="41" t="s">
+      <c r="K6" s="37" t="s">
         <v>228</v>
       </c>
       <c r="M6" s="18">
@@ -1979,7 +1961,7 @@
         <v>10</v>
       </c>
       <c r="J7" s="13"/>
-      <c r="K7" s="41" t="s">
+      <c r="K7" s="37" t="s">
         <v>226</v>
       </c>
       <c r="M7" s="18">
@@ -2045,7 +2027,7 @@
       <c r="J8" s="13">
         <v>41861</v>
       </c>
-      <c r="K8" s="40" t="s">
+      <c r="K8" s="36" t="s">
         <v>227</v>
       </c>
       <c r="M8" s="18">
@@ -2111,7 +2093,7 @@
       <c r="J9" s="13">
         <v>46117</v>
       </c>
-      <c r="K9" s="39" t="s">
+      <c r="K9" s="35" t="s">
         <v>264</v>
       </c>
       <c r="L9" t="s">
@@ -2246,7 +2228,7 @@
       <c r="J11" s="13">
         <v>41861</v>
       </c>
-      <c r="K11" s="40" t="s">
+      <c r="K11" s="36" t="s">
         <v>227</v>
       </c>
       <c r="M11" s="18">
@@ -2312,7 +2294,7 @@
       <c r="J12" s="13">
         <v>41861</v>
       </c>
-      <c r="K12" s="40" t="s">
+      <c r="K12" s="36" t="s">
         <v>227</v>
       </c>
       <c r="M12" s="18">
@@ -2842,7 +2824,7 @@
       <c r="J20" s="13">
         <v>42031</v>
       </c>
-      <c r="K20" s="40" t="s">
+      <c r="K20" s="36" t="s">
         <v>227</v>
       </c>
       <c r="M20" s="18">
@@ -16220,7 +16202,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -16232,10 +16214,10 @@
       <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="36" t="s">
+      <c r="E1" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="36" t="s">
+      <c r="F1" s="39" t="s">
         <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -16243,7 +16225,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="35"/>
+      <c r="A2" s="38"/>
       <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
@@ -16253,8 +16235,8 @@
       <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
       <c r="G2" s="1" t="s">
         <v>8</v>
       </c>
@@ -16401,22 +16383,22 @@
       <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="37">
+      <c r="B9" s="40">
         <v>2.7480000000000002</v>
       </c>
-      <c r="C9" s="37">
+      <c r="C9" s="40">
         <v>3.282</v>
       </c>
-      <c r="D9" s="37">
+      <c r="D9" s="40">
         <v>3.7109999999999999</v>
       </c>
-      <c r="E9" s="38">
+      <c r="E9" s="41">
         <v>12.8</v>
       </c>
-      <c r="F9" s="38">
+      <c r="F9" s="41">
         <v>6.69</v>
       </c>
-      <c r="G9" s="37" t="s">
+      <c r="G9" s="40" t="s">
         <v>10</v>
       </c>
     </row>
@@ -16424,33 +16406,33 @@
       <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="38"/>
-      <c r="F10" s="38"/>
-      <c r="G10" s="37"/>
+      <c r="B10" s="40"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="41"/>
+      <c r="G10" s="40"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="37">
+      <c r="B11" s="40">
         <v>3.665</v>
       </c>
-      <c r="C11" s="37">
+      <c r="C11" s="40">
         <v>5.46</v>
       </c>
-      <c r="D11" s="37">
+      <c r="D11" s="40">
         <v>4.6849999999999996</v>
       </c>
-      <c r="E11" s="38">
+      <c r="E11" s="41">
         <v>18.399999999999999</v>
       </c>
-      <c r="F11" s="38">
+      <c r="F11" s="41">
         <v>8.4499999999999993</v>
       </c>
-      <c r="G11" s="37" t="s">
+      <c r="G11" s="40" t="s">
         <v>10</v>
       </c>
     </row>
@@ -16458,12 +16440,12 @@
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="37"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="38"/>
-      <c r="G12" s="37"/>
+      <c r="B12" s="40"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="40"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
@@ -16607,22 +16589,22 @@
       <c r="A19" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="37">
+      <c r="B19" s="40">
         <v>4.5910000000000002</v>
       </c>
-      <c r="C19" s="37">
+      <c r="C19" s="40">
         <v>9.8949999999999996</v>
       </c>
-      <c r="D19" s="37">
+      <c r="D19" s="40">
         <v>9.0860000000000003</v>
       </c>
-      <c r="E19" s="38">
+      <c r="E19" s="41">
         <v>28.5</v>
       </c>
-      <c r="F19" s="38">
+      <c r="F19" s="41">
         <v>16.399999999999999</v>
       </c>
-      <c r="G19" s="37" t="s">
+      <c r="G19" s="40" t="s">
         <v>10</v>
       </c>
     </row>
@@ -16630,12 +16612,12 @@
       <c r="A20" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="37"/>
-      <c r="C20" s="37"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="38"/>
-      <c r="G20" s="37"/>
+      <c r="B20" s="40"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="40"/>
+      <c r="E20" s="41"/>
+      <c r="F20" s="41"/>
+      <c r="G20" s="40"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
@@ -17259,7 +17241,7 @@
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="35" t="s">
+      <c r="A48" s="38" t="s">
         <v>0</v>
       </c>
       <c r="B48" s="1" t="s">
@@ -17271,10 +17253,10 @@
       <c r="D48" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E48" s="36" t="s">
+      <c r="E48" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="F48" s="36" t="s">
+      <c r="F48" s="39" t="s">
         <v>6</v>
       </c>
       <c r="G48" s="1" t="s">
@@ -17282,7 +17264,7 @@
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="35"/>
+      <c r="A49" s="38"/>
       <c r="B49" s="1" t="s">
         <v>2</v>
       </c>
@@ -17292,14 +17274,30 @@
       <c r="D49" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E49" s="36"/>
-      <c r="F49" s="36"/>
+      <c r="E49" s="39"/>
+      <c r="F49" s="39"/>
       <c r="G49" s="1" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="G11:G12"/>
     <mergeCell ref="A48:A49"/>
     <mergeCell ref="E48:E49"/>
     <mergeCell ref="F48:F49"/>
@@ -17308,22 +17306,6 @@
     <mergeCell ref="D19:D20"/>
     <mergeCell ref="E19:E20"/>
     <mergeCell ref="F19:F20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="F9:F10"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" display="http://pdadb.net/index.php?m=cpu&amp;id=a6422&amp;c=samsung_s5p6422" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
@@ -20330,20 +20312,21 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9DDF9A1-601F-4A84-9995-BE5D51EA74DF}">
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.5703125" customWidth="1"/>
     <col min="2" max="2" width="23.28515625" customWidth="1"/>
     <col min="3" max="3" width="6.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.140625" customWidth="1"/>
-    <col min="5" max="6" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.140625" customWidth="1"/>
+    <col min="9" max="9" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A1" s="42" t="s">
         <v>78</v>
       </c>
@@ -20357,55 +20340,62 @@
         <v>80</v>
       </c>
       <c r="E1" s="43" t="s">
-        <v>81</v>
+        <v>268</v>
       </c>
       <c r="F1" s="43" t="s">
         <v>82</v>
       </c>
       <c r="G1" s="43" t="s">
+        <v>181</v>
+      </c>
+      <c r="H1" s="43" t="s">
+        <v>238</v>
+      </c>
+      <c r="I1" s="43" t="s">
         <v>83</v>
       </c>
-      <c r="H1" s="43" t="s">
-        <v>181</v>
-      </c>
-      <c r="I1" s="43" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="46" t="s">
+      <c r="K1" s="43" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="44" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="44" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="44">
+      <c r="C2" s="45">
         <v>667</v>
       </c>
-      <c r="D2" s="44">
+      <c r="D2" s="45">
         <v>0.54100000000000004</v>
       </c>
-      <c r="E2" s="44">
+      <c r="E2" s="45" t="str">
+        <f>CONCATENATE("__", K2, "__")</f>
+        <v>__0.959__</v>
+      </c>
+      <c r="F2" s="45">
+        <v>0.126</v>
+      </c>
+      <c r="G2" s="46">
+        <v>40892</v>
+      </c>
+      <c r="H2" s="45" t="s">
+        <v>228</v>
+      </c>
+      <c r="I2" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="45">
         <v>0.95899999999999996</v>
       </c>
-      <c r="F2" s="44">
-        <v>0.126</v>
-      </c>
-      <c r="G2" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" s="48">
-        <v>40892</v>
-      </c>
-      <c r="I2" s="44" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="47" t="s">
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="44" t="s">
         <v>92</v>
       </c>
-      <c r="B3" s="47" t="s">
+      <c r="B3" s="44" t="s">
         <v>148</v>
       </c>
       <c r="C3" s="45">
@@ -20414,56 +20404,64 @@
       <c r="D3" s="45">
         <v>1.238</v>
       </c>
-      <c r="E3" s="45">
-        <v>1.33</v>
+      <c r="E3" s="45" t="str">
+        <f t="shared" ref="E3:E60" si="0">CONCATENATE("__", K3, "__")</f>
+        <v>__1.33__</v>
       </c>
       <c r="F3" s="45">
         <v>2.4089999999999998</v>
       </c>
-      <c r="G3" s="45" t="s">
+      <c r="G3" s="46">
+        <v>41122</v>
+      </c>
+      <c r="H3" s="45" t="s">
+        <v>225</v>
+      </c>
+      <c r="I3" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="49">
-        <v>41122</v>
-      </c>
-      <c r="I3" s="45" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="46" t="s">
+      <c r="K3" s="45">
+        <v>1.33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="44" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="44" t="s">
         <v>146</v>
       </c>
-      <c r="C4" s="44">
+      <c r="C4" s="45">
         <v>600</v>
       </c>
-      <c r="D4" s="44">
+      <c r="D4" s="45">
         <v>1.04</v>
       </c>
-      <c r="E4" s="44">
+      <c r="E4" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__1.685__</v>
+      </c>
+      <c r="F4" s="45">
+        <v>0.22800000000000001</v>
+      </c>
+      <c r="G4" s="46">
+        <v>41487</v>
+      </c>
+      <c r="H4" s="45" t="s">
+        <v>228</v>
+      </c>
+      <c r="I4" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="K4" s="45">
         <v>1.6850000000000001</v>
       </c>
-      <c r="F4" s="44">
-        <v>0.22800000000000001</v>
-      </c>
-      <c r="G4" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H4" s="48">
-        <v>41487</v>
-      </c>
-      <c r="I4" s="44" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="47" t="s">
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="44" t="s">
         <v>90</v>
       </c>
-      <c r="B5" s="47" t="s">
+      <c r="B5" s="44" t="s">
         <v>91</v>
       </c>
       <c r="C5" s="45">
@@ -20472,56 +20470,64 @@
       <c r="D5" s="45">
         <v>1.379</v>
       </c>
-      <c r="E5" s="45">
-        <v>1.712</v>
+      <c r="E5" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__1.712__</v>
       </c>
       <c r="F5" s="45">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="G5" s="45" t="s">
+      <c r="G5" s="46">
+        <v>41489</v>
+      </c>
+      <c r="H5" s="45" t="s">
+        <v>229</v>
+      </c>
+      <c r="I5" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="49">
-        <v>41489</v>
-      </c>
-      <c r="I5" s="45" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="46" t="s">
+      <c r="K5" s="45">
+        <v>1.712</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="44" t="s">
         <v>88</v>
       </c>
-      <c r="B6" s="46" t="s">
+      <c r="B6" s="44" t="s">
         <v>147</v>
       </c>
-      <c r="C6" s="44">
+      <c r="C6" s="45">
         <v>667</v>
       </c>
-      <c r="D6" s="44">
+      <c r="D6" s="45">
         <v>1.024</v>
       </c>
-      <c r="E6" s="44">
+      <c r="E6" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__1.821__</v>
+      </c>
+      <c r="F6" s="45">
+        <v>0.23799999999999999</v>
+      </c>
+      <c r="G6" s="46">
+        <v>41122</v>
+      </c>
+      <c r="H6" s="45" t="s">
+        <v>228</v>
+      </c>
+      <c r="I6" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="K6" s="45">
         <v>1.821</v>
       </c>
-      <c r="F6" s="44">
-        <v>0.23799999999999999</v>
-      </c>
-      <c r="G6" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H6" s="48">
-        <v>41122</v>
-      </c>
-      <c r="I6" s="44" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="47" t="s">
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="44" t="s">
         <v>89</v>
       </c>
-      <c r="B7" s="47" t="s">
+      <c r="B7" s="44" t="s">
         <v>93</v>
       </c>
       <c r="C7" s="45">
@@ -20530,54 +20536,62 @@
       <c r="D7" s="45">
         <v>2.456</v>
       </c>
-      <c r="E7" s="45">
-        <v>3.1059999999999999</v>
+      <c r="E7" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__3.106__</v>
       </c>
       <c r="F7" s="45">
         <v>2.0289999999999999</v>
       </c>
-      <c r="G7" s="45" t="s">
+      <c r="G7" s="46"/>
+      <c r="H7" s="45" t="s">
+        <v>226</v>
+      </c>
+      <c r="I7" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="H7" s="49"/>
-      <c r="I7" s="45" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="46" t="s">
+      <c r="K7" s="45">
+        <v>3.1059999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="44" t="s">
         <v>95</v>
       </c>
-      <c r="B8" s="46" t="s">
+      <c r="B8" s="44" t="s">
         <v>143</v>
       </c>
-      <c r="C8" s="44">
+      <c r="C8" s="45">
         <v>800</v>
       </c>
-      <c r="D8" s="44">
+      <c r="D8" s="45">
         <v>2.7480000000000002</v>
       </c>
-      <c r="E8" s="44">
+      <c r="E8" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__3.282__</v>
+      </c>
+      <c r="F8" s="45">
+        <v>3.7109999999999999</v>
+      </c>
+      <c r="G8" s="46">
+        <v>41861</v>
+      </c>
+      <c r="H8" s="45" t="s">
+        <v>227</v>
+      </c>
+      <c r="I8" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="K8" s="45">
         <v>3.282</v>
       </c>
-      <c r="F8" s="44">
-        <v>3.7109999999999999</v>
-      </c>
-      <c r="G8" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H8" s="48">
-        <v>41861</v>
-      </c>
-      <c r="I8" s="44" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="47" t="s">
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="44" t="s">
         <v>265</v>
       </c>
-      <c r="B9" s="47" t="s">
+      <c r="B9" s="44" t="s">
         <v>266</v>
       </c>
       <c r="C9" s="45">
@@ -20586,56 +20600,64 @@
       <c r="D9" s="45">
         <v>1.7330000000000001</v>
       </c>
-      <c r="E9" s="45">
-        <v>3.9889999999999999</v>
+      <c r="E9" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__3.989__</v>
       </c>
       <c r="F9" s="45">
         <v>0.25</v>
       </c>
-      <c r="G9" s="45" t="s">
+      <c r="G9" s="46">
+        <v>46117</v>
+      </c>
+      <c r="H9" s="45" t="s">
+        <v>264</v>
+      </c>
+      <c r="I9" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="49">
-        <v>46117</v>
-      </c>
-      <c r="I9" s="45" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="46" t="s">
+      <c r="K9" s="45">
+        <v>3.9889999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="44" t="s">
         <v>96</v>
       </c>
-      <c r="B10" s="46" t="s">
+      <c r="B10" s="44" t="s">
         <v>159</v>
       </c>
-      <c r="C10" s="44">
+      <c r="C10" s="45">
         <v>933</v>
       </c>
-      <c r="D10" s="44">
+      <c r="D10" s="45">
         <v>4.7089999999999996</v>
       </c>
-      <c r="E10" s="44">
+      <c r="E10" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__5.164__</v>
+      </c>
+      <c r="F10" s="45">
+        <v>8.9160000000000004</v>
+      </c>
+      <c r="G10" s="46">
+        <v>41861</v>
+      </c>
+      <c r="H10" s="45" t="s">
+        <v>225</v>
+      </c>
+      <c r="I10" s="45" t="s">
+        <v>22</v>
+      </c>
+      <c r="K10" s="45">
         <v>5.1639999999999997</v>
       </c>
-      <c r="F10" s="44">
-        <v>8.9160000000000004</v>
-      </c>
-      <c r="G10" s="44" t="s">
-        <v>22</v>
-      </c>
-      <c r="H10" s="48">
-        <v>41861</v>
-      </c>
-      <c r="I10" s="44" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="47" t="s">
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="44" t="s">
         <v>94</v>
       </c>
-      <c r="B11" s="47" t="s">
+      <c r="B11" s="44" t="s">
         <v>144</v>
       </c>
       <c r="C11" s="45">
@@ -20644,56 +20666,64 @@
       <c r="D11" s="45">
         <v>3.665</v>
       </c>
-      <c r="E11" s="45">
-        <v>5.46</v>
+      <c r="E11" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__5.46__</v>
       </c>
       <c r="F11" s="45">
         <v>4.6849999999999996</v>
       </c>
-      <c r="G11" s="45" t="s">
+      <c r="G11" s="46">
+        <v>41861</v>
+      </c>
+      <c r="H11" s="45" t="s">
+        <v>227</v>
+      </c>
+      <c r="I11" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="H11" s="49">
+      <c r="K11" s="45">
+        <v>5.46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="44" t="s">
+        <v>97</v>
+      </c>
+      <c r="B12" s="44" t="s">
+        <v>115</v>
+      </c>
+      <c r="C12" s="45">
+        <v>1000</v>
+      </c>
+      <c r="D12" s="45">
+        <v>4.665</v>
+      </c>
+      <c r="E12" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__6.481__</v>
+      </c>
+      <c r="F12" s="45">
+        <v>5.0590000000000002</v>
+      </c>
+      <c r="G12" s="46">
         <v>41861</v>
       </c>
-      <c r="I11" s="45" t="s">
+      <c r="H12" s="45" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="46" t="s">
-        <v>97</v>
-      </c>
-      <c r="B12" s="46" t="s">
-        <v>115</v>
-      </c>
-      <c r="C12" s="44">
-        <v>1000</v>
-      </c>
-      <c r="D12" s="44">
-        <v>4.665</v>
-      </c>
-      <c r="E12" s="44">
+      <c r="I12" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="K12" s="45">
         <v>6.4809999999999999</v>
       </c>
-      <c r="F12" s="44">
-        <v>5.0590000000000002</v>
-      </c>
-      <c r="G12" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H12" s="48">
-        <v>41861</v>
-      </c>
-      <c r="I12" s="44" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="47" t="s">
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="44" t="s">
         <v>99</v>
       </c>
-      <c r="B13" s="47" t="s">
+      <c r="B13" s="44" t="s">
         <v>116</v>
       </c>
       <c r="C13" s="45">
@@ -20702,56 +20732,64 @@
       <c r="D13" s="45">
         <v>5.7990000000000004</v>
       </c>
-      <c r="E13" s="45">
-        <v>6.7169999999999996</v>
+      <c r="E13" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__6.717__</v>
       </c>
       <c r="F13" s="45">
         <v>8.0549999999999997</v>
       </c>
-      <c r="G13" s="45" t="s">
+      <c r="G13" s="46">
+        <v>42217</v>
+      </c>
+      <c r="H13" s="45" t="s">
+        <v>224</v>
+      </c>
+      <c r="I13" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="49">
-        <v>42217</v>
-      </c>
-      <c r="I13" s="45" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="46" t="s">
+      <c r="K13" s="45">
+        <v>6.7169999999999996</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="44" t="s">
         <v>98</v>
       </c>
-      <c r="B14" s="46" t="s">
+      <c r="B14" s="44" t="s">
         <v>117</v>
       </c>
-      <c r="C14" s="44">
+      <c r="C14" s="45">
         <v>1200</v>
       </c>
-      <c r="D14" s="44">
+      <c r="D14" s="45">
         <v>6.21</v>
       </c>
-      <c r="E14" s="44">
+      <c r="E14" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__7.047__</v>
+      </c>
+      <c r="F14" s="45">
+        <v>12.384</v>
+      </c>
+      <c r="G14" s="46">
+        <v>41797</v>
+      </c>
+      <c r="H14" s="45" t="s">
+        <v>225</v>
+      </c>
+      <c r="I14" s="45" t="s">
+        <v>26</v>
+      </c>
+      <c r="K14" s="45">
         <v>7.0469999999999997</v>
       </c>
-      <c r="F14" s="44">
-        <v>12.384</v>
-      </c>
-      <c r="G14" s="44" t="s">
-        <v>26</v>
-      </c>
-      <c r="H14" s="48">
-        <v>41797</v>
-      </c>
-      <c r="I14" s="44" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="47" t="s">
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="44" t="s">
         <v>153</v>
       </c>
-      <c r="B15" s="47" t="s">
+      <c r="B15" s="44" t="s">
         <v>119</v>
       </c>
       <c r="C15" s="45">
@@ -20760,56 +20798,64 @@
       <c r="D15" s="45">
         <v>7.2430000000000003</v>
       </c>
-      <c r="E15" s="45">
-        <v>7.109</v>
+      <c r="E15" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__7.109__</v>
       </c>
       <c r="F15" s="45">
         <v>7.351</v>
       </c>
-      <c r="G15" s="45" t="s">
+      <c r="G15" s="46">
+        <v>40269</v>
+      </c>
+      <c r="H15" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I15" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="H15" s="49">
-        <v>40269</v>
-      </c>
-      <c r="I15" s="45" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="46" t="s">
+      <c r="K15" s="45">
+        <v>7.109</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="44" t="s">
         <v>154</v>
       </c>
-      <c r="B16" s="46" t="s">
+      <c r="B16" s="44" t="s">
         <v>102</v>
       </c>
-      <c r="C16" s="44">
+      <c r="C16" s="45">
         <v>2000</v>
       </c>
-      <c r="D16" s="44">
+      <c r="D16" s="45">
         <v>9.3940000000000001</v>
       </c>
-      <c r="E16" s="44">
+      <c r="E16" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__7.529__</v>
+      </c>
+      <c r="F16" s="45">
+        <v>13.164</v>
+      </c>
+      <c r="G16" s="46">
+        <v>40017</v>
+      </c>
+      <c r="H16" s="45" t="s">
+        <v>225</v>
+      </c>
+      <c r="I16" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="K16" s="45">
         <v>7.5289999999999999</v>
       </c>
-      <c r="F16" s="44">
-        <v>13.164</v>
-      </c>
-      <c r="G16" s="44" t="s">
-        <v>35</v>
-      </c>
-      <c r="H16" s="48">
-        <v>40017</v>
-      </c>
-      <c r="I16" s="44" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="47" t="s">
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="44" t="s">
         <v>149</v>
       </c>
-      <c r="B17" s="47" t="s">
+      <c r="B17" s="44" t="s">
         <v>118</v>
       </c>
       <c r="C17" s="45">
@@ -20818,56 +20864,64 @@
       <c r="D17" s="45">
         <v>7.7519999999999998</v>
       </c>
-      <c r="E17" s="45">
-        <v>7.5789999999999997</v>
+      <c r="E17" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__7.579__</v>
       </c>
       <c r="F17" s="45">
         <v>7.0679999999999996</v>
       </c>
-      <c r="G17" s="45" t="s">
+      <c r="G17" s="46">
+        <v>40026</v>
+      </c>
+      <c r="H17" s="45" t="s">
+        <v>225</v>
+      </c>
+      <c r="I17" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="H17" s="49">
-        <v>40026</v>
-      </c>
-      <c r="I17" s="45" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="46" t="s">
+      <c r="K17" s="45">
+        <v>7.5789999999999997</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="44" t="s">
         <v>155</v>
       </c>
-      <c r="B18" s="46" t="s">
+      <c r="B18" s="44" t="s">
         <v>101</v>
       </c>
-      <c r="C18" s="44">
+      <c r="C18" s="45">
         <v>1666</v>
       </c>
-      <c r="D18" s="44">
+      <c r="D18" s="45">
         <v>9.3859999999999992</v>
       </c>
-      <c r="E18" s="44">
+      <c r="E18" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__8.39__</v>
+      </c>
+      <c r="F18" s="45">
+        <v>7.3129999999999997</v>
+      </c>
+      <c r="G18" s="46">
+        <v>41496</v>
+      </c>
+      <c r="H18" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I18" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="K18" s="45">
         <v>8.39</v>
       </c>
-      <c r="F18" s="44">
-        <v>7.3129999999999997</v>
-      </c>
-      <c r="G18" s="44" t="s">
-        <v>33</v>
-      </c>
-      <c r="H18" s="48">
-        <v>41496</v>
-      </c>
-      <c r="I18" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="47" t="s">
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="44" t="s">
         <v>214</v>
       </c>
-      <c r="B19" s="47" t="s">
+      <c r="B19" s="44" t="s">
         <v>215</v>
       </c>
       <c r="C19" s="45">
@@ -20876,56 +20930,64 @@
       <c r="D19" s="45">
         <v>6.78</v>
       </c>
-      <c r="E19" s="45">
-        <v>9.5239999999999991</v>
+      <c r="E19" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__9.524__</v>
       </c>
       <c r="F19" s="45">
         <v>9.1739999999999995</v>
       </c>
-      <c r="G19" s="45" t="s">
+      <c r="G19" s="46">
+        <v>45298</v>
+      </c>
+      <c r="H19" s="45" t="s">
+        <v>224</v>
+      </c>
+      <c r="I19" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="H19" s="49">
-        <v>45298</v>
-      </c>
-      <c r="I19" s="45" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="46" t="s">
+      <c r="K19" s="45">
+        <v>9.5239999999999991</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="44" t="s">
         <v>100</v>
       </c>
-      <c r="B20" s="46" t="s">
+      <c r="B20" s="44" t="s">
         <v>145</v>
       </c>
-      <c r="C20" s="44">
+      <c r="C20" s="45">
         <v>1512</v>
       </c>
-      <c r="D20" s="44">
+      <c r="D20" s="45">
         <v>4.5910000000000002</v>
       </c>
-      <c r="E20" s="44">
+      <c r="E20" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__9.895__</v>
+      </c>
+      <c r="F20" s="45">
+        <v>9.0860000000000003</v>
+      </c>
+      <c r="G20" s="46">
+        <v>42031</v>
+      </c>
+      <c r="H20" s="45" t="s">
+        <v>227</v>
+      </c>
+      <c r="I20" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="K20" s="45">
         <v>9.8949999999999996</v>
       </c>
-      <c r="F20" s="44">
-        <v>9.0860000000000003</v>
-      </c>
-      <c r="G20" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H20" s="48">
-        <v>42031</v>
-      </c>
-      <c r="I20" s="44" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="47" t="s">
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="44" t="s">
         <v>182</v>
       </c>
-      <c r="B21" s="47" t="s">
+      <c r="B21" s="44" t="s">
         <v>183</v>
       </c>
       <c r="C21" s="45">
@@ -20934,56 +20996,64 @@
       <c r="D21" s="45">
         <v>8.68</v>
       </c>
-      <c r="E21" s="45">
-        <v>10.948</v>
+      <c r="E21" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__10.948__</v>
       </c>
       <c r="F21" s="45">
         <v>10.154999999999999</v>
       </c>
-      <c r="G21" s="45" t="s">
+      <c r="G21" s="46">
+        <v>45319</v>
+      </c>
+      <c r="H21" s="45" t="s">
+        <v>224</v>
+      </c>
+      <c r="I21" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="H21" s="49">
-        <v>45319</v>
-      </c>
-      <c r="I21" s="45" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="46" t="s">
+      <c r="K21" s="45">
+        <v>10.948</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="44" t="s">
         <v>111</v>
       </c>
-      <c r="B22" s="46" t="s">
+      <c r="B22" s="44" t="s">
         <v>103</v>
       </c>
-      <c r="C22" s="44">
+      <c r="C22" s="45">
         <v>1800</v>
       </c>
-      <c r="D22" s="44">
+      <c r="D22" s="45">
         <v>11.269</v>
       </c>
-      <c r="E22" s="44">
+      <c r="E22" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__11.927__</v>
+      </c>
+      <c r="F22" s="45">
+        <v>20.516999999999999</v>
+      </c>
+      <c r="G22" s="46">
+        <v>40672</v>
+      </c>
+      <c r="H22" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I22" s="45" t="s">
+        <v>187</v>
+      </c>
+      <c r="K22" s="45">
         <v>11.927</v>
       </c>
-      <c r="F22" s="44">
-        <v>20.516999999999999</v>
-      </c>
-      <c r="G22" s="44" t="s">
-        <v>187</v>
-      </c>
-      <c r="H22" s="48">
-        <v>40672</v>
-      </c>
-      <c r="I22" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="47" t="s">
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="44" t="s">
         <v>156</v>
       </c>
-      <c r="B23" s="47" t="s">
+      <c r="B23" s="44" t="s">
         <v>104</v>
       </c>
       <c r="C23" s="45">
@@ -20992,56 +21062,64 @@
       <c r="D23" s="45">
         <v>12.138</v>
       </c>
-      <c r="E23" s="45">
-        <v>12.568</v>
+      <c r="E23" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__12.568__</v>
       </c>
       <c r="F23" s="45">
         <v>21.143999999999998</v>
       </c>
-      <c r="G23" s="45" t="s">
+      <c r="G23" s="46">
+        <v>39919</v>
+      </c>
+      <c r="H23" s="45" t="s">
+        <v>225</v>
+      </c>
+      <c r="I23" s="45" t="s">
         <v>188</v>
       </c>
-      <c r="H23" s="49">
-        <v>39919</v>
-      </c>
-      <c r="I23" s="45" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="46" t="s">
+      <c r="K23" s="45">
+        <v>12.568</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="44" t="s">
         <v>158</v>
       </c>
-      <c r="B24" s="46" t="s">
+      <c r="B24" s="44" t="s">
         <v>106</v>
       </c>
-      <c r="C24" s="44">
+      <c r="C24" s="45">
         <v>1860</v>
       </c>
-      <c r="D24" s="44">
+      <c r="D24" s="45">
         <v>18.433</v>
       </c>
-      <c r="E24" s="44">
+      <c r="E24" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__15.15__</v>
+      </c>
+      <c r="F24" s="45">
+        <v>16.635999999999999</v>
+      </c>
+      <c r="G24" s="46">
+        <v>41788</v>
+      </c>
+      <c r="H24" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I24" s="45" t="s">
+        <v>189</v>
+      </c>
+      <c r="K24" s="45">
         <v>15.15</v>
       </c>
-      <c r="F24" s="44">
-        <v>16.635999999999999</v>
-      </c>
-      <c r="G24" s="44" t="s">
-        <v>189</v>
-      </c>
-      <c r="H24" s="48">
-        <v>41788</v>
-      </c>
-      <c r="I24" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="47" t="s">
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="44" t="s">
         <v>231</v>
       </c>
-      <c r="B25" s="47" t="s">
+      <c r="B25" s="44" t="s">
         <v>232</v>
       </c>
       <c r="C25" s="45">
@@ -21050,54 +21128,62 @@
       <c r="D25" s="45">
         <v>14.398999999999999</v>
       </c>
-      <c r="E25" s="45">
-        <v>15.946999999999999</v>
+      <c r="E25" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__15.947__</v>
       </c>
       <c r="F25" s="45">
         <v>17.788</v>
       </c>
-      <c r="G25" s="45"/>
-      <c r="H25" s="49">
+      <c r="G25" s="46">
         <v>45772</v>
       </c>
-      <c r="I25" s="45" t="s">
+      <c r="H25" s="45" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="46" t="s">
+      <c r="I25" s="45"/>
+      <c r="K25" s="45">
+        <v>15.946999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="44" t="s">
         <v>111</v>
       </c>
-      <c r="B26" s="46" t="s">
+      <c r="B26" s="44" t="s">
         <v>160</v>
       </c>
-      <c r="C26" s="44">
+      <c r="C26" s="45">
         <v>1800</v>
       </c>
-      <c r="D26" s="44">
+      <c r="D26" s="45">
         <v>13.595000000000001</v>
       </c>
-      <c r="E26" s="44">
+      <c r="E26" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__16.121__</v>
+      </c>
+      <c r="F26" s="45">
+        <v>19.565999999999999</v>
+      </c>
+      <c r="G26" s="46">
+        <v>40672</v>
+      </c>
+      <c r="H26" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I26" s="45" t="s">
+        <v>190</v>
+      </c>
+      <c r="K26" s="45">
         <v>16.120999999999999</v>
       </c>
-      <c r="F26" s="44">
-        <v>19.565999999999999</v>
-      </c>
-      <c r="G26" s="44" t="s">
-        <v>190</v>
-      </c>
-      <c r="H26" s="48">
-        <v>40672</v>
-      </c>
-      <c r="I26" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="47" t="s">
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" s="44" t="s">
         <v>161</v>
       </c>
-      <c r="B27" s="47" t="s">
+      <c r="B27" s="44" t="s">
         <v>107</v>
       </c>
       <c r="C27" s="45">
@@ -21106,56 +21192,64 @@
       <c r="D27" s="45">
         <v>19.981000000000002</v>
       </c>
-      <c r="E27" s="45">
-        <v>16.207000000000001</v>
+      <c r="E27" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__16.207__</v>
       </c>
       <c r="F27" s="45">
         <v>18.001000000000001</v>
       </c>
-      <c r="G27" s="45" t="s">
+      <c r="G27" s="46">
+        <v>41851</v>
+      </c>
+      <c r="H27" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I27" s="45" t="s">
         <v>191</v>
       </c>
-      <c r="H27" s="49">
-        <v>41851</v>
-      </c>
-      <c r="I27" s="45" t="s">
+      <c r="K27" s="45">
+        <v>16.207000000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="44" t="s">
+        <v>112</v>
+      </c>
+      <c r="B28" s="44" t="s">
+        <v>122</v>
+      </c>
+      <c r="C28" s="45">
+        <v>1299</v>
+      </c>
+      <c r="D28" s="45">
+        <v>19.050999999999998</v>
+      </c>
+      <c r="E28" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__17.286__</v>
+      </c>
+      <c r="F28" s="45">
+        <v>25.289000000000001</v>
+      </c>
+      <c r="G28" s="46">
+        <v>41861</v>
+      </c>
+      <c r="H28" s="45" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="46" t="s">
-        <v>112</v>
-      </c>
-      <c r="B28" s="46" t="s">
-        <v>122</v>
-      </c>
-      <c r="C28" s="44">
-        <v>1299</v>
-      </c>
-      <c r="D28" s="44">
-        <v>19.050999999999998</v>
-      </c>
-      <c r="E28" s="44">
+      <c r="I28" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="K28" s="45">
         <v>17.286000000000001</v>
       </c>
-      <c r="F28" s="44">
-        <v>25.289000000000001</v>
-      </c>
-      <c r="G28" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H28" s="48">
-        <v>41861</v>
-      </c>
-      <c r="I28" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="47" t="s">
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="44" t="s">
         <v>137</v>
       </c>
-      <c r="B29" s="47" t="s">
+      <c r="B29" s="44" t="s">
         <v>110</v>
       </c>
       <c r="C29" s="45">
@@ -21164,56 +21258,64 @@
       <c r="D29" s="45">
         <v>28.488</v>
       </c>
-      <c r="E29" s="45">
-        <v>17.780999999999999</v>
+      <c r="E29" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__17.781__</v>
       </c>
       <c r="F29" s="45">
         <v>36.673000000000002</v>
       </c>
-      <c r="G29" s="45" t="s">
+      <c r="G29" s="46">
+        <v>41457</v>
+      </c>
+      <c r="H29" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I29" s="45" t="s">
         <v>192</v>
       </c>
-      <c r="H29" s="49">
-        <v>41457</v>
-      </c>
-      <c r="I29" s="45" t="s">
+      <c r="K29" s="45">
+        <v>17.780999999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="44" t="s">
+        <v>113</v>
+      </c>
+      <c r="B30" s="44" t="s">
+        <v>123</v>
+      </c>
+      <c r="C30" s="45">
+        <v>1600</v>
+      </c>
+      <c r="D30" s="45">
+        <v>23.695</v>
+      </c>
+      <c r="E30" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__17.817__</v>
+      </c>
+      <c r="F30" s="45">
+        <v>25.515999999999998</v>
+      </c>
+      <c r="G30" s="46">
+        <v>44089</v>
+      </c>
+      <c r="H30" s="45" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="46" t="s">
-        <v>113</v>
-      </c>
-      <c r="B30" s="46" t="s">
-        <v>123</v>
-      </c>
-      <c r="C30" s="44">
-        <v>1600</v>
-      </c>
-      <c r="D30" s="44">
-        <v>23.695</v>
-      </c>
-      <c r="E30" s="44">
+      <c r="I30" s="45" t="s">
+        <v>210</v>
+      </c>
+      <c r="K30" s="45">
         <v>17.817</v>
       </c>
-      <c r="F30" s="44">
-        <v>25.515999999999998</v>
-      </c>
-      <c r="G30" s="44" t="s">
-        <v>210</v>
-      </c>
-      <c r="H30" s="48">
-        <v>44089</v>
-      </c>
-      <c r="I30" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="47" t="s">
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="44" t="s">
         <v>108</v>
       </c>
-      <c r="B31" s="47" t="s">
+      <c r="B31" s="44" t="s">
         <v>121</v>
       </c>
       <c r="C31" s="45">
@@ -21222,56 +21324,64 @@
       <c r="D31" s="45">
         <v>18.776</v>
       </c>
-      <c r="E31" s="45">
-        <v>17.878</v>
+      <c r="E31" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__17.878__</v>
       </c>
       <c r="F31" s="45">
         <v>29.106000000000002</v>
       </c>
-      <c r="G31" s="45" t="s">
+      <c r="G31" s="46">
+        <v>43641</v>
+      </c>
+      <c r="H31" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I31" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="H31" s="49">
-        <v>43641</v>
-      </c>
-      <c r="I31" s="45" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="46" t="s">
+      <c r="K31" s="45">
+        <v>17.878</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="44" t="s">
         <v>212</v>
       </c>
-      <c r="B32" s="46" t="s">
+      <c r="B32" s="44" t="s">
         <v>213</v>
       </c>
-      <c r="C32" s="44">
+      <c r="C32" s="45">
         <v>1500</v>
       </c>
-      <c r="D32" s="44">
+      <c r="D32" s="45">
         <v>15.319000000000001</v>
       </c>
-      <c r="E32" s="44">
+      <c r="E32" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__18.061__</v>
+      </c>
+      <c r="F32" s="45">
+        <v>34.619999999999997</v>
+      </c>
+      <c r="G32" s="46">
+        <v>45561</v>
+      </c>
+      <c r="H32" s="45" t="s">
+        <v>224</v>
+      </c>
+      <c r="I32" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="K32" s="45">
         <v>18.061</v>
       </c>
-      <c r="F32" s="44">
-        <v>34.619999999999997</v>
-      </c>
-      <c r="G32" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H32" s="48">
-        <v>45561</v>
-      </c>
-      <c r="I32" s="44" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="47" t="s">
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="44" t="s">
         <v>162</v>
       </c>
-      <c r="B33" s="47" t="s">
+      <c r="B33" s="44" t="s">
         <v>109</v>
       </c>
       <c r="C33" s="45">
@@ -21280,56 +21390,64 @@
       <c r="D33" s="45">
         <v>18.265000000000001</v>
       </c>
-      <c r="E33" s="45">
-        <v>18.957999999999998</v>
+      <c r="E33" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__18.958__</v>
       </c>
       <c r="F33" s="45">
         <v>31.843</v>
       </c>
-      <c r="G33" s="45" t="s">
+      <c r="G33" s="46">
+        <v>41151</v>
+      </c>
+      <c r="H33" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I33" s="45" t="s">
         <v>193</v>
       </c>
-      <c r="H33" s="49">
-        <v>41151</v>
-      </c>
-      <c r="I33" s="45" t="s">
+      <c r="K33" s="45">
+        <v>18.957999999999998</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="44" t="s">
+        <v>157</v>
+      </c>
+      <c r="B34" s="44" t="s">
+        <v>105</v>
+      </c>
+      <c r="C34" s="45">
+        <v>2100</v>
+      </c>
+      <c r="D34" s="45">
+        <v>14.395</v>
+      </c>
+      <c r="E34" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__19.299__</v>
+      </c>
+      <c r="F34" s="45">
+        <v>23.132000000000001</v>
+      </c>
+      <c r="G34" s="46">
+        <v>40060</v>
+      </c>
+      <c r="H34" s="45" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="46" t="s">
-        <v>157</v>
-      </c>
-      <c r="B34" s="46" t="s">
-        <v>105</v>
-      </c>
-      <c r="C34" s="44">
-        <v>2100</v>
-      </c>
-      <c r="D34" s="44">
-        <v>14.395</v>
-      </c>
-      <c r="E34" s="44">
+      <c r="I34" s="45" t="s">
+        <v>43</v>
+      </c>
+      <c r="K34" s="45">
         <v>19.298999999999999</v>
       </c>
-      <c r="F34" s="44">
-        <v>23.132000000000001</v>
-      </c>
-      <c r="G34" s="44" t="s">
-        <v>43</v>
-      </c>
-      <c r="H34" s="48">
-        <v>40060</v>
-      </c>
-      <c r="I34" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="47" t="s">
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="44" t="s">
         <v>136</v>
       </c>
-      <c r="B35" s="47" t="s">
+      <c r="B35" s="44" t="s">
         <v>134</v>
       </c>
       <c r="C35" s="45">
@@ -21338,56 +21456,64 @@
       <c r="D35" s="45">
         <v>28.631</v>
       </c>
-      <c r="E35" s="45">
-        <v>19.780999999999999</v>
+      <c r="E35" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__19.781__</v>
       </c>
       <c r="F35" s="45">
         <v>31.140999999999998</v>
       </c>
-      <c r="G35" s="45" t="s">
+      <c r="G35" s="46">
+        <v>42713</v>
+      </c>
+      <c r="H35" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I35" s="45" t="s">
         <v>206</v>
       </c>
-      <c r="H35" s="49">
-        <v>42713</v>
-      </c>
-      <c r="I35" s="45" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="46" t="s">
+      <c r="K35" s="45">
+        <v>19.780999999999999</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="44" t="s">
         <v>245</v>
       </c>
-      <c r="B36" s="46" t="s">
+      <c r="B36" s="44" t="s">
         <v>247</v>
       </c>
-      <c r="C36" s="44">
+      <c r="C36" s="45">
         <v>2400</v>
       </c>
-      <c r="D36" s="44">
+      <c r="D36" s="45">
         <v>23.448</v>
       </c>
-      <c r="E36" s="44">
+      <c r="E36" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__32.408__</v>
+      </c>
+      <c r="F36" s="45">
+        <v>50.741999999999997</v>
+      </c>
+      <c r="G36" s="46">
+        <v>46116</v>
+      </c>
+      <c r="H36" s="45" t="s">
+        <v>224</v>
+      </c>
+      <c r="I36" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="K36" s="45">
         <v>32.408000000000001</v>
       </c>
-      <c r="F36" s="44">
-        <v>50.741999999999997</v>
-      </c>
-      <c r="G36" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H36" s="48">
-        <v>46116</v>
-      </c>
-      <c r="I36" s="44" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="47" t="s">
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="44" t="s">
         <v>163</v>
       </c>
-      <c r="B37" s="47" t="s">
+      <c r="B37" s="44" t="s">
         <v>164</v>
       </c>
       <c r="C37" s="45">
@@ -21396,56 +21522,64 @@
       <c r="D37" s="45">
         <v>19.359000000000002</v>
       </c>
-      <c r="E37" s="45">
-        <v>19.808</v>
+      <c r="E37" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__19.808__</v>
       </c>
       <c r="F37" s="45">
         <v>33.182000000000002</v>
       </c>
-      <c r="G37" s="45" t="s">
+      <c r="G37" s="46">
+        <v>41919</v>
+      </c>
+      <c r="H37" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I37" s="45" t="s">
         <v>205</v>
       </c>
-      <c r="H37" s="49">
-        <v>41919</v>
-      </c>
-      <c r="I37" s="45" t="s">
+      <c r="K37" s="45">
+        <v>19.808</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" s="44" t="s">
+        <v>135</v>
+      </c>
+      <c r="B38" s="44" t="s">
+        <v>133</v>
+      </c>
+      <c r="C38" s="45">
+        <v>2832</v>
+      </c>
+      <c r="D38" s="45">
+        <v>33.670999999999999</v>
+      </c>
+      <c r="E38" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__23.584__</v>
+      </c>
+      <c r="F38" s="45">
+        <v>36.384</v>
+      </c>
+      <c r="G38" s="46">
+        <v>42443</v>
+      </c>
+      <c r="H38" s="45" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="46" t="s">
-        <v>135</v>
-      </c>
-      <c r="B38" s="46" t="s">
-        <v>133</v>
-      </c>
-      <c r="C38" s="44">
-        <v>2832</v>
-      </c>
-      <c r="D38" s="44">
-        <v>33.670999999999999</v>
-      </c>
-      <c r="E38" s="44">
+      <c r="I38" s="45" t="s">
+        <v>204</v>
+      </c>
+      <c r="K38" s="45">
         <v>23.584</v>
       </c>
-      <c r="F38" s="44">
-        <v>36.384</v>
-      </c>
-      <c r="G38" s="44" t="s">
-        <v>204</v>
-      </c>
-      <c r="H38" s="48">
-        <v>42443</v>
-      </c>
-      <c r="I38" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="47" t="s">
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" s="44" t="s">
         <v>174</v>
       </c>
-      <c r="B39" s="47" t="s">
+      <c r="B39" s="44" t="s">
         <v>175</v>
       </c>
       <c r="C39" s="45">
@@ -21454,56 +21588,64 @@
       <c r="D39" s="45">
         <v>28.776</v>
       </c>
-      <c r="E39" s="45">
-        <v>23.881</v>
+      <c r="E39" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__23.881__</v>
       </c>
       <c r="F39" s="45">
         <v>47.396000000000001</v>
       </c>
-      <c r="G39" s="45" t="s">
+      <c r="G39" s="46">
+        <v>44691</v>
+      </c>
+      <c r="H39" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I39" s="45" t="s">
         <v>203</v>
       </c>
-      <c r="H39" s="49">
-        <v>44691</v>
-      </c>
-      <c r="I39" s="45" t="s">
+      <c r="K39" s="45">
+        <v>23.881</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" s="44" t="s">
+        <v>150</v>
+      </c>
+      <c r="B40" s="44" t="s">
+        <v>131</v>
+      </c>
+      <c r="C40" s="45">
+        <v>3200</v>
+      </c>
+      <c r="D40" s="45">
+        <v>37.845999999999997</v>
+      </c>
+      <c r="E40" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__23.882__</v>
+      </c>
+      <c r="F40" s="45">
+        <v>47.436999999999998</v>
+      </c>
+      <c r="G40" s="46">
+        <v>41537</v>
+      </c>
+      <c r="H40" s="45" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="46" t="s">
-        <v>150</v>
-      </c>
-      <c r="B40" s="46" t="s">
-        <v>131</v>
-      </c>
-      <c r="C40" s="44">
-        <v>3200</v>
-      </c>
-      <c r="D40" s="44">
-        <v>37.845999999999997</v>
-      </c>
-      <c r="E40" s="44">
+      <c r="I40" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="K40" s="45">
         <v>23.882000000000001</v>
       </c>
-      <c r="F40" s="44">
-        <v>47.436999999999998</v>
-      </c>
-      <c r="G40" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H40" s="48">
-        <v>41537</v>
-      </c>
-      <c r="I40" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="47" t="s">
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" s="44" t="s">
         <v>151</v>
       </c>
-      <c r="B41" s="47" t="s">
+      <c r="B41" s="44" t="s">
         <v>132</v>
       </c>
       <c r="C41" s="45">
@@ -21512,56 +21654,64 @@
       <c r="D41" s="45">
         <v>24.206</v>
       </c>
-      <c r="E41" s="45">
-        <v>24.602</v>
+      <c r="E41" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__24.602__</v>
       </c>
       <c r="F41" s="45">
         <v>41.085000000000001</v>
       </c>
-      <c r="G41" s="45" t="s">
+      <c r="G41" s="46">
+        <v>40683</v>
+      </c>
+      <c r="H41" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I41" s="45" t="s">
         <v>202</v>
       </c>
-      <c r="H41" s="49">
-        <v>40683</v>
-      </c>
-      <c r="I41" s="45" t="s">
+      <c r="K41" s="45">
+        <v>24.602</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" s="44" t="s">
+        <v>186</v>
+      </c>
+      <c r="B42" s="44" t="s">
+        <v>114</v>
+      </c>
+      <c r="C42" s="45">
+        <v>2829</v>
+      </c>
+      <c r="D42" s="45">
+        <v>21.475999999999999</v>
+      </c>
+      <c r="E42" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__25.608__</v>
+      </c>
+      <c r="F42" s="45">
+        <v>30.663</v>
+      </c>
+      <c r="G42" s="46">
+        <v>39896</v>
+      </c>
+      <c r="H42" s="45" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="46" t="s">
-        <v>186</v>
-      </c>
-      <c r="B42" s="46" t="s">
-        <v>114</v>
-      </c>
-      <c r="C42" s="44">
-        <v>2829</v>
-      </c>
-      <c r="D42" s="44">
-        <v>21.475999999999999</v>
-      </c>
-      <c r="E42" s="44">
+      <c r="I42" s="45" t="s">
+        <v>201</v>
+      </c>
+      <c r="K42" s="45">
         <v>25.608000000000001</v>
       </c>
-      <c r="F42" s="44">
-        <v>30.663</v>
-      </c>
-      <c r="G42" s="44" t="s">
-        <v>201</v>
-      </c>
-      <c r="H42" s="48">
-        <v>39896</v>
-      </c>
-      <c r="I42" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="47" t="s">
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" s="44" t="s">
         <v>167</v>
       </c>
-      <c r="B43" s="47" t="s">
+      <c r="B43" s="44" t="s">
         <v>168</v>
       </c>
       <c r="C43" s="45">
@@ -21570,56 +21720,64 @@
       <c r="D43" s="45">
         <v>27.460999999999999</v>
       </c>
-      <c r="E43" s="45">
-        <v>26.341999999999999</v>
+      <c r="E43" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__26.342__</v>
       </c>
       <c r="F43" s="45">
         <v>27.893999999999998</v>
       </c>
-      <c r="G43" s="45" t="s">
+      <c r="G43" s="46">
+        <v>43956</v>
+      </c>
+      <c r="H43" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I43" s="45" t="s">
         <v>211</v>
       </c>
-      <c r="H43" s="49">
-        <v>43956</v>
-      </c>
-      <c r="I43" s="45" t="s">
+      <c r="K43" s="45">
+        <v>26.341999999999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" s="44" t="s">
+        <v>138</v>
+      </c>
+      <c r="B44" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="C44" s="45">
+        <v>3352</v>
+      </c>
+      <c r="D44" s="45">
+        <v>28.021999999999998</v>
+      </c>
+      <c r="E44" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__32.586__</v>
+      </c>
+      <c r="F44" s="45">
+        <v>44.103999999999999</v>
+      </c>
+      <c r="G44" s="46">
+        <v>42315</v>
+      </c>
+      <c r="H44" s="45" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="46" t="s">
-        <v>138</v>
-      </c>
-      <c r="B44" s="46" t="s">
-        <v>130</v>
-      </c>
-      <c r="C44" s="44">
-        <v>3352</v>
-      </c>
-      <c r="D44" s="44">
-        <v>28.021999999999998</v>
-      </c>
-      <c r="E44" s="44">
+      <c r="I44" s="45" t="s">
+        <v>200</v>
+      </c>
+      <c r="K44" s="45">
         <v>32.585999999999999</v>
       </c>
-      <c r="F44" s="44">
-        <v>44.103999999999999</v>
-      </c>
-      <c r="G44" s="44" t="s">
-        <v>200</v>
-      </c>
-      <c r="H44" s="48">
-        <v>42315</v>
-      </c>
-      <c r="I44" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="47" t="s">
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" s="44" t="s">
         <v>120</v>
       </c>
-      <c r="B45" s="47" t="s">
+      <c r="B45" s="44" t="s">
         <v>171</v>
       </c>
       <c r="C45" s="45">
@@ -21628,56 +21786,64 @@
       <c r="D45" s="45">
         <v>39.049999999999997</v>
       </c>
-      <c r="E45" s="45">
-        <v>33.215000000000003</v>
+      <c r="E45" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__33.215__</v>
       </c>
       <c r="F45" s="45">
         <v>54.26</v>
       </c>
-      <c r="G45" s="45" t="s">
+      <c r="G45" s="46">
+        <v>42397</v>
+      </c>
+      <c r="H45" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I45" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="H45" s="49">
+      <c r="K45" s="45">
+        <v>33.215000000000003</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" s="44" t="s">
+        <v>139</v>
+      </c>
+      <c r="B46" s="44" t="s">
+        <v>140</v>
+      </c>
+      <c r="C46" s="45">
+        <v>2500</v>
+      </c>
+      <c r="D46" s="45">
+        <v>40.698999999999998</v>
+      </c>
+      <c r="E46" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__37.018__</v>
+      </c>
+      <c r="F46" s="45">
+        <v>52.634999999999998</v>
+      </c>
+      <c r="G46" s="46">
         <v>42397</v>
       </c>
-      <c r="I45" s="45" t="s">
+      <c r="H46" s="45" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="46" t="s">
-        <v>139</v>
-      </c>
-      <c r="B46" s="46" t="s">
-        <v>140</v>
-      </c>
-      <c r="C46" s="44">
-        <v>2500</v>
-      </c>
-      <c r="D46" s="44">
-        <v>40.698999999999998</v>
-      </c>
-      <c r="E46" s="44">
+      <c r="I46" s="45" t="s">
+        <v>199</v>
+      </c>
+      <c r="K46" s="45">
         <v>37.018000000000001</v>
       </c>
-      <c r="F46" s="44">
-        <v>52.634999999999998</v>
-      </c>
-      <c r="G46" s="44" t="s">
-        <v>199</v>
-      </c>
-      <c r="H46" s="48">
-        <v>42397</v>
-      </c>
-      <c r="I46" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="47" t="s">
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="B47" s="47" t="s">
+      <c r="B47" s="44" t="s">
         <v>142</v>
       </c>
       <c r="C47" s="45">
@@ -21686,56 +21852,64 @@
       <c r="D47" s="45">
         <v>45.381999999999998</v>
       </c>
-      <c r="E47" s="45">
-        <v>40.313000000000002</v>
+      <c r="E47" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__40.313__</v>
       </c>
       <c r="F47" s="45">
         <v>61.804000000000002</v>
       </c>
-      <c r="G47" s="45" t="s">
+      <c r="G47" s="46">
+        <v>42817</v>
+      </c>
+      <c r="H47" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I47" s="45" t="s">
         <v>198</v>
       </c>
-      <c r="H47" s="49">
-        <v>42817</v>
-      </c>
-      <c r="I47" s="45" t="s">
+      <c r="K47" s="45">
+        <v>40.313000000000002</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A48" s="44" t="s">
+        <v>173</v>
+      </c>
+      <c r="B48" s="44" t="s">
+        <v>166</v>
+      </c>
+      <c r="C48" s="45">
+        <v>2700</v>
+      </c>
+      <c r="D48" s="45">
+        <v>57.2</v>
+      </c>
+      <c r="E48" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__43.732__</v>
+      </c>
+      <c r="F48" s="45">
+        <v>107.95399999999999</v>
+      </c>
+      <c r="G48" s="46">
+        <v>44155</v>
+      </c>
+      <c r="H48" s="45" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="46" t="s">
-        <v>173</v>
-      </c>
-      <c r="B48" s="46" t="s">
-        <v>166</v>
-      </c>
-      <c r="C48" s="44">
-        <v>2700</v>
-      </c>
-      <c r="D48" s="44">
-        <v>57.2</v>
-      </c>
-      <c r="E48" s="44">
+      <c r="I48" s="45" t="s">
+        <v>197</v>
+      </c>
+      <c r="K48" s="45">
         <v>43.731999999999999</v>
       </c>
-      <c r="F48" s="44">
-        <v>107.95399999999999</v>
-      </c>
-      <c r="G48" s="44" t="s">
-        <v>197</v>
-      </c>
-      <c r="H48" s="48">
-        <v>44155</v>
-      </c>
-      <c r="I48" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="47" t="s">
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" s="44" t="s">
         <v>127</v>
       </c>
-      <c r="B49" s="47" t="s">
+      <c r="B49" s="44" t="s">
         <v>172</v>
       </c>
       <c r="C49" s="45">
@@ -21744,56 +21918,64 @@
       <c r="D49" s="45">
         <v>55.045999999999999</v>
       </c>
-      <c r="E49" s="45">
-        <v>44.618000000000002</v>
+      <c r="E49" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__44.618__</v>
       </c>
       <c r="F49" s="45">
         <v>73.569999999999993</v>
       </c>
-      <c r="G49" s="45" t="s">
+      <c r="G49" s="46">
+        <v>43355</v>
+      </c>
+      <c r="H49" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I49" s="45" t="s">
         <v>196</v>
       </c>
-      <c r="H49" s="49">
-        <v>43355</v>
-      </c>
-      <c r="I49" s="45" t="s">
+      <c r="K49" s="45">
+        <v>44.618000000000002</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" s="44" t="s">
+        <v>126</v>
+      </c>
+      <c r="B50" s="44" t="s">
+        <v>124</v>
+      </c>
+      <c r="C50" s="45">
+        <v>2600</v>
+      </c>
+      <c r="D50" s="45">
+        <v>63.682000000000002</v>
+      </c>
+      <c r="E50" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__45.732__</v>
+      </c>
+      <c r="F50" s="45">
+        <v>68.159000000000006</v>
+      </c>
+      <c r="G50" s="46">
+        <v>43146</v>
+      </c>
+      <c r="H50" s="45" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" s="46" t="s">
-        <v>126</v>
-      </c>
-      <c r="B50" s="46" t="s">
-        <v>124</v>
-      </c>
-      <c r="C50" s="44">
-        <v>2600</v>
-      </c>
-      <c r="D50" s="44">
-        <v>63.682000000000002</v>
-      </c>
-      <c r="E50" s="44">
+      <c r="I50" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="K50" s="45">
         <v>45.731999999999999</v>
       </c>
-      <c r="F50" s="44">
-        <v>68.159000000000006</v>
-      </c>
-      <c r="G50" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H50" s="48">
-        <v>43146</v>
-      </c>
-      <c r="I50" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A51" s="47" t="s">
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" s="44" t="s">
         <v>128</v>
       </c>
-      <c r="B51" s="47" t="s">
+      <c r="B51" s="44" t="s">
         <v>125</v>
       </c>
       <c r="C51" s="45">
@@ -21802,56 +21984,64 @@
       <c r="D51" s="45">
         <v>50.423000000000002</v>
       </c>
-      <c r="E51" s="45">
-        <v>46.116999999999997</v>
+      <c r="E51" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__46.117__</v>
       </c>
       <c r="F51" s="45">
         <v>70.039000000000001</v>
       </c>
-      <c r="G51" s="45" t="s">
+      <c r="G51" s="46">
+        <v>43146</v>
+      </c>
+      <c r="H51" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I51" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="H51" s="49">
-        <v>43146</v>
-      </c>
-      <c r="I51" s="45" t="s">
+      <c r="K51" s="45">
+        <v>46.116999999999997</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A52" s="44" t="s">
+        <v>216</v>
+      </c>
+      <c r="B52" s="44" t="s">
+        <v>217</v>
+      </c>
+      <c r="C52" s="45">
+        <v>2112</v>
+      </c>
+      <c r="D52" s="45">
+        <v>61.249000000000002</v>
+      </c>
+      <c r="E52" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__46.227__</v>
+      </c>
+      <c r="F52" s="45">
+        <v>113.619</v>
+      </c>
+      <c r="G52" s="46">
+        <v>45298</v>
+      </c>
+      <c r="H52" s="45" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="46" t="s">
-        <v>216</v>
-      </c>
-      <c r="B52" s="46" t="s">
-        <v>217</v>
-      </c>
-      <c r="C52" s="44">
-        <v>2112</v>
-      </c>
-      <c r="D52" s="44">
-        <v>61.249000000000002</v>
-      </c>
-      <c r="E52" s="44">
+      <c r="I52" s="45" t="s">
+        <v>218</v>
+      </c>
+      <c r="K52" s="45">
         <v>46.226999999999997</v>
       </c>
-      <c r="F52" s="44">
-        <v>113.619</v>
-      </c>
-      <c r="G52" s="44" t="s">
-        <v>218</v>
-      </c>
-      <c r="H52" s="48">
-        <v>45298</v>
-      </c>
-      <c r="I52" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A53" s="47" t="s">
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" s="44" t="s">
         <v>236</v>
       </c>
-      <c r="B53" s="47" t="s">
+      <c r="B53" s="44" t="s">
         <v>237</v>
       </c>
       <c r="C53" s="45">
@@ -21860,54 +22050,62 @@
       <c r="D53" s="45">
         <v>68.150000000000006</v>
       </c>
-      <c r="E53" s="45">
-        <v>48.103000000000002</v>
+      <c r="E53" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__48.103__</v>
       </c>
       <c r="F53" s="45">
         <v>118.447</v>
       </c>
-      <c r="G53" s="45"/>
-      <c r="H53" s="49">
+      <c r="G53" s="46">
         <v>45773</v>
       </c>
-      <c r="I53" s="45" t="s">
+      <c r="H53" s="45" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A54" s="46" t="s">
+      <c r="I53" s="45"/>
+      <c r="K53" s="45">
+        <v>48.103000000000002</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A54" s="44" t="s">
         <v>234</v>
       </c>
-      <c r="B54" s="46" t="s">
+      <c r="B54" s="44" t="s">
         <v>233</v>
       </c>
-      <c r="C54" s="44">
+      <c r="C54" s="45">
         <v>2295</v>
       </c>
-      <c r="D54" s="44">
+      <c r="D54" s="45">
         <v>59.665999999999997</v>
       </c>
-      <c r="E54" s="44">
+      <c r="E54" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__49.441__</v>
+      </c>
+      <c r="F54" s="45">
+        <v>116.922</v>
+      </c>
+      <c r="G54" s="46">
+        <v>45298</v>
+      </c>
+      <c r="H54" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I54" s="45" t="s">
+        <v>235</v>
+      </c>
+      <c r="K54" s="45">
         <v>49.441000000000003</v>
       </c>
-      <c r="F54" s="44">
-        <v>116.922</v>
-      </c>
-      <c r="G54" s="44" t="s">
-        <v>235</v>
-      </c>
-      <c r="H54" s="48">
-        <v>45298</v>
-      </c>
-      <c r="I54" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A55" s="47" t="s">
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A55" s="44" t="s">
         <v>208</v>
       </c>
-      <c r="B55" s="47" t="s">
+      <c r="B55" s="44" t="s">
         <v>209</v>
       </c>
       <c r="C55" s="45">
@@ -21916,83 +22114,95 @@
       <c r="D55" s="45">
         <v>62.206000000000003</v>
       </c>
-      <c r="E55" s="45">
-        <v>49.951000000000001</v>
+      <c r="E55" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__49.951__</v>
       </c>
       <c r="F55" s="45">
         <v>112.593</v>
       </c>
-      <c r="G55" s="45" t="s">
+      <c r="G55" s="46">
+        <v>45561</v>
+      </c>
+      <c r="H55" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I55" s="45" t="s">
         <v>207</v>
       </c>
-      <c r="H55" s="49">
-        <v>45561</v>
-      </c>
-      <c r="I55" s="45" t="s">
+      <c r="K55" s="45">
+        <v>49.951000000000001</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A56" s="44" t="s">
+        <v>177</v>
+      </c>
+      <c r="B56" s="44" t="s">
+        <v>178</v>
+      </c>
+      <c r="C56" s="45">
+        <v>4160</v>
+      </c>
+      <c r="D56" s="45">
+        <v>77.174000000000007</v>
+      </c>
+      <c r="E56" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__56.761__</v>
+      </c>
+      <c r="F56" s="45">
+        <v>138.00299999999999</v>
+      </c>
+      <c r="G56" s="46">
+        <v>45211</v>
+      </c>
+      <c r="H56" s="45" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A56" s="46" t="s">
-        <v>177</v>
-      </c>
-      <c r="B56" s="46" t="s">
-        <v>178</v>
-      </c>
-      <c r="C56" s="44">
-        <v>4160</v>
-      </c>
-      <c r="D56" s="44">
-        <v>77.174000000000007</v>
-      </c>
-      <c r="E56" s="44">
+      <c r="I56" s="45" t="s">
+        <v>195</v>
+      </c>
+      <c r="K56" s="45">
         <v>56.761000000000003</v>
       </c>
-      <c r="F56" s="44">
-        <v>138.00299999999999</v>
-      </c>
-      <c r="G56" s="44" t="s">
-        <v>195</v>
-      </c>
-      <c r="H56" s="48">
-        <v>45211</v>
-      </c>
-      <c r="I56" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A57" s="46" t="s">
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A57" s="44" t="s">
         <v>246</v>
       </c>
-      <c r="B57" s="46" t="s">
+      <c r="B57" s="44" t="s">
         <v>249</v>
       </c>
-      <c r="C57" s="44">
+      <c r="C57" s="45">
         <v>3090</v>
       </c>
-      <c r="D57" s="44">
+      <c r="D57" s="45">
         <v>63.435000000000002</v>
       </c>
-      <c r="E57" s="44">
+      <c r="E57" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__66.735__</v>
+      </c>
+      <c r="F57" s="45">
+        <v>143.465</v>
+      </c>
+      <c r="G57" s="46">
+        <v>46116</v>
+      </c>
+      <c r="H57" s="45" t="s">
+        <v>250</v>
+      </c>
+      <c r="I57" s="45"/>
+      <c r="K57" s="45">
         <v>66.734999999999999</v>
       </c>
-      <c r="F57" s="44">
-        <v>143.465</v>
-      </c>
-      <c r="G57" s="44"/>
-      <c r="H57" s="48">
-        <v>46116</v>
-      </c>
-      <c r="I57" s="44" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A58" s="47" t="s">
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A58" s="44" t="s">
         <v>220</v>
       </c>
-      <c r="B58" s="47" t="s">
+      <c r="B58" s="44" t="s">
         <v>219</v>
       </c>
       <c r="C58" s="45">
@@ -22001,56 +22211,64 @@
       <c r="D58" s="45">
         <v>66.938999999999993</v>
       </c>
-      <c r="E58" s="45">
-        <v>79.733000000000004</v>
+      <c r="E58" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__79.733__</v>
       </c>
       <c r="F58" s="45">
         <v>216.304</v>
       </c>
-      <c r="G58" s="45" t="s">
+      <c r="G58" s="46">
+        <v>45561</v>
+      </c>
+      <c r="H58" s="45" t="s">
+        <v>230</v>
+      </c>
+      <c r="I58" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="H58" s="49">
+      <c r="K58" s="45">
+        <v>79.733000000000004</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A59" s="44" t="s">
+        <v>184</v>
+      </c>
+      <c r="B59" s="44" t="s">
+        <v>185</v>
+      </c>
+      <c r="C59" s="45">
+        <v>4700</v>
+      </c>
+      <c r="D59" s="45">
+        <v>104.52500000000001</v>
+      </c>
+      <c r="E59" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__85.011__</v>
+      </c>
+      <c r="F59" s="45">
+        <v>264.86900000000003</v>
+      </c>
+      <c r="G59" s="46">
         <v>45561</v>
       </c>
-      <c r="I58" s="45" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A59" s="46" t="s">
-        <v>184</v>
-      </c>
-      <c r="B59" s="46" t="s">
-        <v>185</v>
-      </c>
-      <c r="C59" s="44">
-        <v>4700</v>
-      </c>
-      <c r="D59" s="44">
-        <v>104.52500000000001</v>
-      </c>
-      <c r="E59" s="44">
-        <v>85.01</v>
-      </c>
-      <c r="F59" s="44">
-        <v>264.86900000000003</v>
-      </c>
-      <c r="G59" s="44" t="s">
+      <c r="H59" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="I59" s="45" t="s">
         <v>194</v>
       </c>
-      <c r="H59" s="48">
-        <v>45561</v>
-      </c>
-      <c r="I59" s="44" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A60" s="47" t="s">
+      <c r="K59" s="45">
+        <v>85.010999999999996</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A60" s="44" t="s">
         <v>253</v>
       </c>
-      <c r="B60" s="47" t="s">
+      <c r="B60" s="44" t="s">
         <v>254</v>
       </c>
       <c r="C60" s="45">
@@ -22059,49 +22277,53 @@
       <c r="D60" s="45">
         <v>83.274000000000001</v>
       </c>
-      <c r="E60" s="45">
-        <v>86</v>
+      <c r="E60" s="45" t="str">
+        <f t="shared" si="0"/>
+        <v>__86.001__</v>
       </c>
       <c r="F60" s="45">
         <v>163.31299999999999</v>
       </c>
-      <c r="G60" s="45" t="s">
+      <c r="G60" s="46">
+        <v>46116</v>
+      </c>
+      <c r="H60" s="45" t="s">
+        <v>255</v>
+      </c>
+      <c r="I60" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="H60" s="49">
-        <v>46116</v>
-      </c>
-      <c r="I60" s="45" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="K60" s="45">
+        <v>86.001000000000005</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A61" s="42" t="s">
         <v>78</v>
       </c>
       <c r="B61" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C61" s="44" t="s">
+      <c r="C61" s="45" t="s">
         <v>84</v>
       </c>
-      <c r="D61" s="44" t="s">
+      <c r="D61" s="45" t="s">
         <v>80</v>
       </c>
       <c r="E61" s="43" t="s">
         <v>81</v>
       </c>
-      <c r="F61" s="44" t="s">
+      <c r="F61" s="45" t="s">
         <v>82</v>
       </c>
-      <c r="G61" s="44" t="s">
+      <c r="G61" s="43" t="s">
+        <v>181</v>
+      </c>
+      <c r="H61" s="45" t="s">
+        <v>238</v>
+      </c>
+      <c r="I61" s="45" t="s">
         <v>83</v>
-      </c>
-      <c r="H61" s="43" t="s">
-        <v>181</v>
-      </c>
-      <c r="I61" s="44" t="s">
-        <v>238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>